<commit_message>
run all tests for conlusion testing
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData2.xlsx
+++ b/src/test/resources/testdata/TestData2.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6800" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>username</t>
   </si>
@@ -37,10 +37,13 @@
     <t>password</t>
   </si>
   <si>
-    <t>Admin</t>
+    <t>orangehrm_chaker</t>
   </si>
   <si>
-    <t>admin123</t>
+    <t>AdminOrangeHRM12@!</t>
+  </si>
+  <si>
+    <t>AdminOrangeHRM12@!!</t>
   </si>
   <si>
     <t>emp_id</t>
@@ -665,11 +668,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1200,46 +1209,49 @@
   <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="15.9090909090909" customWidth="1"/>
-    <col min="2" max="2" width="14.2727272727273" customWidth="1"/>
+    <col min="1" max="1" width="19.0909090909091" customWidth="1"/>
+    <col min="2" max="2" width="23.3636363636364" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="2" customFormat="1" spans="1:2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:2">
-      <c r="A2" s="1" t="s">
+    <row r="2" s="2" customFormat="1" spans="1:2">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1"/>
-    <row r="4" s="1" customFormat="1"/>
-    <row r="5" s="1" customFormat="1"/>
-    <row r="6" s="1" customFormat="1"/>
-    <row r="7" s="1" customFormat="1"/>
-    <row r="8" s="1" customFormat="1"/>
-    <row r="9" s="1" customFormat="1"/>
-    <row r="10" s="1" customFormat="1"/>
-    <row r="11" s="1" customFormat="1"/>
-    <row r="12" s="1" customFormat="1"/>
-    <row r="13" s="1" customFormat="1"/>
-    <row r="14" s="1" customFormat="1"/>
-    <row r="15" s="1" customFormat="1"/>
-    <row r="16" s="1" customFormat="1"/>
-    <row r="17" s="1" customFormat="1"/>
-    <row r="18" s="1" customFormat="1"/>
-    <row r="19" s="1" customFormat="1"/>
-    <row r="20" s="1" customFormat="1"/>
-    <row r="21" s="1" customFormat="1"/>
+    <row r="3" s="2" customFormat="1"/>
+    <row r="4" s="2" customFormat="1"/>
+    <row r="5" s="2" customFormat="1"/>
+    <row r="6" s="2" customFormat="1"/>
+    <row r="7" s="2" customFormat="1"/>
+    <row r="8" s="2" customFormat="1"/>
+    <row r="9" s="2" customFormat="1"/>
+    <row r="10" s="2" customFormat="1"/>
+    <row r="11" s="2" customFormat="1"/>
+    <row r="12" s="2" customFormat="1"/>
+    <row r="13" s="2" customFormat="1"/>
+    <row r="14" s="2" customFormat="1"/>
+    <row r="15" s="2" customFormat="1"/>
+    <row r="16" s="2" customFormat="1"/>
+    <row r="17" s="2" customFormat="1"/>
+    <row r="18" s="2" customFormat="1"/>
+    <row r="19" s="2" customFormat="1"/>
+    <row r="20" s="2" customFormat="1"/>
+    <row r="21" s="2" customFormat="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="AdminOrangeHRM12@!"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1251,24 +1263,82 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="15.9090909090909" customWidth="1"/>
-    <col min="2" max="2" width="14.2727272727273" customWidth="1"/>
+    <col min="1" max="1" width="18.8181818181818" customWidth="1"/>
+    <col min="2" max="2" width="21.9090909090909" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="2" customFormat="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" s="2" customFormat="1" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" s="2" customFormat="1"/>
+    <row r="4" s="2" customFormat="1"/>
+    <row r="5" s="2" customFormat="1"/>
+    <row r="6" s="2" customFormat="1"/>
+    <row r="7" s="2" customFormat="1"/>
+    <row r="8" s="2" customFormat="1"/>
+    <row r="9" s="2" customFormat="1"/>
+    <row r="10" s="2" customFormat="1"/>
+    <row r="11" s="2" customFormat="1"/>
+    <row r="12" s="2" customFormat="1"/>
+    <row r="13" s="2" customFormat="1"/>
+    <row r="14" s="2" customFormat="1"/>
+    <row r="15" s="2" customFormat="1"/>
+    <row r="16" s="2" customFormat="1"/>
+    <row r="17" s="2" customFormat="1"/>
+    <row r="18" s="2" customFormat="1"/>
+    <row r="19" s="2" customFormat="1"/>
+    <row r="20" s="2" customFormat="1"/>
+    <row r="21" s="2" customFormat="1"/>
+    <row r="22" s="2" customFormat="1"/>
+    <row r="23" s="2" customFormat="1"/>
+    <row r="24" s="2" customFormat="1"/>
+    <row r="25" s="2" customFormat="1"/>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="AdminOrangeHRM12@!!"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B41"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="15.0909090909091" customWidth="1"/>
+    <col min="2" max="2" width="15.8181818181818" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" spans="1:2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="1">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1"/>
@@ -1294,38 +1364,22 @@
     <row r="23" s="1" customFormat="1"/>
     <row r="24" s="1" customFormat="1"/>
     <row r="25" s="1" customFormat="1"/>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1"/>
-  <cols>
-    <col min="1" max="1" width="15.0909090909091" customWidth="1"/>
-    <col min="2" max="2" width="15.8181818181818" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-    </row>
+    <row r="26" s="1" customFormat="1"/>
+    <row r="27" s="1" customFormat="1"/>
+    <row r="28" s="1" customFormat="1"/>
+    <row r="29" s="1" customFormat="1"/>
+    <row r="30" s="1" customFormat="1"/>
+    <row r="31" s="1" customFormat="1"/>
+    <row r="32" s="1" customFormat="1"/>
+    <row r="33" s="1" customFormat="1"/>
+    <row r="34" s="1" customFormat="1"/>
+    <row r="35" s="1" customFormat="1"/>
+    <row r="36" s="1" customFormat="1"/>
+    <row r="37" s="1" customFormat="1"/>
+    <row r="38" s="1" customFormat="1"/>
+    <row r="39" s="1" customFormat="1"/>
+    <row r="40" s="1" customFormat="1"/>
+    <row r="41" s="1" customFormat="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>